<commit_message>
PPWR Compliance Suite v1.0.0 — İnci Akü tam ürün.
Müşteri arayüzü Türkçe; teslimat setleri programa bağlı; Render için disk ve giriş hazır.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/candidates/PPWR_CANDIDATE_DELIVERY_REV00/00_CONTROL/INCI_PPWR_CANDIDATE_ENGINE_Rev00.xlsx
+++ b/candidates/PPWR_CANDIDATE_DELIVERY_REV00/00_CONTROL/INCI_PPWR_CANDIDATE_ENGINE_Rev00.xlsx
@@ -524,7 +524,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Candidates only  •  Rev.00 draft  •  Publish 11.08.2026  •  2026-08-17 14:08 UTC</t>
+          <t>Candidates only  •  Rev.00 draft  •  Publish 11.08.2026  •  2026-08-18 11:11 UTC</t>
         </is>
       </c>
     </row>
@@ -806,12 +806,12 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>CAND_DEMO01</t>
+          <t>1000069</t>
         </is>
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>AKU,C-FLAT,DK,200AH,INCI SUPRA SENTOR</t>
+          <t>AKÜ,C-FLAT,DK,200AH,İNCİ SUPRA SENTOR</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
@@ -944,12 +944,12 @@
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>CAND_DEMO01</t>
+          <t>1000069</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>AKU,C-FLAT,DK,200AH,INCI SUPRA SENTOR</t>
+          <t>AKÜ,C-FLAT,DK,200AH,İNCİ SUPRA SENTOR</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
@@ -968,35 +968,35 @@
         </is>
       </c>
       <c r="F5" s="13">
-        <f>HYPERLINK("..\01_PRODUCTS\CAND_DEMO01\01_Technical_File.docx","OPEN WORD")</f>
+        <f>HYPERLINK("..\01_PRODUCTS\1000069\01_Technical_File.docx","OPEN WORD")</f>
         <v/>
       </c>
       <c r="G5" s="13">
-        <f>HYPERLINK("..\01_PRODUCTS\CAND_DEMO01\01_Technical_File.pdf","OPEN PDF")</f>
+        <f>HYPERLINK("..\01_PRODUCTS\1000069\01_Technical_File.pdf","OPEN PDF")</f>
         <v/>
       </c>
       <c r="H5" s="13">
-        <f>HYPERLINK("..\01_PRODUCTS\CAND_DEMO01\02_EU_DoC.docx","OPEN WORD")</f>
+        <f>HYPERLINK("..\01_PRODUCTS\1000069\02_EU_DoC.docx","OPEN WORD")</f>
         <v/>
       </c>
       <c r="I5" s="13">
-        <f>HYPERLINK("..\01_PRODUCTS\CAND_DEMO01\02_EU_DoC.pdf","OPEN PDF")</f>
+        <f>HYPERLINK("..\01_PRODUCTS\1000069\02_EU_DoC.pdf","OPEN PDF")</f>
         <v/>
       </c>
       <c r="J5" s="13">
-        <f>HYPERLINK("..\01_PRODUCTS\CAND_DEMO01\03_Label.docx","OPEN WORD")</f>
+        <f>HYPERLINK("..\01_PRODUCTS\1000069\03_Label.docx","OPEN WORD")</f>
         <v/>
       </c>
       <c r="K5" s="13">
-        <f>HYPERLINK("..\01_PRODUCTS\CAND_DEMO01\03_Label.pdf","OPEN PDF")</f>
+        <f>HYPERLINK("..\01_PRODUCTS\1000069\03_Label.pdf","OPEN PDF")</f>
         <v/>
       </c>
       <c r="L5" s="13">
-        <f>HYPERLINK("..\01_PRODUCTS\CAND_DEMO01\04_Shipment_Statement.docx","OPEN WORD")</f>
+        <f>HYPERLINK("..\01_PRODUCTS\1000069\04_Shipment_Statement.docx","OPEN WORD")</f>
         <v/>
       </c>
       <c r="M5" s="13">
-        <f>HYPERLINK("..\01_PRODUCTS\CAND_DEMO01\04_Shipment_Statement.pdf","OPEN PDF")</f>
+        <f>HYPERLINK("..\01_PRODUCTS\1000069\04_Shipment_Statement.pdf","OPEN PDF")</f>
         <v/>
       </c>
     </row>

</xml_diff>